<commit_message>
adding more to checklist
</commit_message>
<xml_diff>
--- a/dspackagefolder/template/checklist/GENERIC_CHECKLIST.xlsx
+++ b/dspackagefolder/template/checklist/GENERIC_CHECKLIST.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rajim\Desktop\NonPHD_Muizdeen\INTERVIEWS\dspackage\dspackagefolder\template\checklist\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80E41AF2-2A65-4CB2-B9DA-DC6EAE93E2B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E0FDF65-9BC9-4E56-8E5E-4C03CD20369F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,9 +25,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
   <si>
     <t>check about 10 digits from the output of the analysis and ensure you can manually generate such numbers and they have been dq-ed</t>
+  </si>
+  <si>
+    <t>CHECKLIST</t>
   </si>
 </sst>
 </file>
@@ -72,7 +75,17 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="3">
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -83,6 +96,16 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{65C1E661-4582-4641-86AB-3C6FE5EE6E5A}" name="Table1" displayName="Table1" ref="A1:A1048576" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
+  <autoFilter ref="A1:A1048576" xr:uid="{65C1E661-4582-4641-86AB-3C6FE5EE6E5A}"/>
+  <tableColumns count="1">
+    <tableColumn id="1" xr3:uid="{25BD2411-6041-4738-B1D5-AE3022ADC147}" name="CHECKLIST" dataDxfId="2"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -348,12 +371,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2"/>
+  <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="55.1796875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
     <row r="2" spans="1:1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>0</v>
@@ -361,5 +389,8 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>